<commit_message>
N-PORT Security: the Proving Run passed; quality check; approval
The one Proving Run (13F, then N-PORT by CUSIP, then by ISIN): 423,562
Securities, 0 CUSIPs and 0 ISINs on two Securities, the second pass
changed nothing. An issuer name filed as a stand-in is withheld (0
records in this quarter). Rules approved under the operator's standing
words; switch-on and merge wait for the operator.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XffcaJSmoXmrPyZxCeFHRa
</commit_message>
<xml_diff>
--- a/rules/sources/sec.nport.security/MAPPING.xlsx
+++ b/rules/sources/sec.nport.security/MAPPING.xlsx
@@ -1079,16 +1079,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:G3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="15" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="62" customWidth="1" min="4" max="4"/>
+    <col width="23" customWidth="1" min="5" max="5"/>
+    <col width="51" customWidth="1" min="6" max="6"/>
+    <col width="46" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1125,6 +1125,80 @@
       <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Rules path</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>sec.nport.security.v1</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>placeholder_name_of_issuer</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Check</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>The value is not a placeholder: NONE, NULL, UNKNOWN, TBD, NOTAPPLICABLE, NOTAVAILABLE</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>fields.name_of_issuer</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Withheld: kept on the record, never used to match</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>quality.sec.nport.security.v1.checks[0]</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>sec.nport.security_isin.v1</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>placeholder_name_of_issuer</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Check</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>The value is not a placeholder: NONE, NULL, UNKNOWN, TBD, NOTAPPLICABLE, NOTAVAILABLE</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>fields.name_of_issuer</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Withheld: kept on the record, never used to match</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>quality.sec.nport.security_isin.v1.checks[0]</t>
         </is>
       </c>
     </row>
@@ -1432,7 +1506,7 @@
           <t>rules file comment</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr"/>
+      <c r="D2" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Ticket 102: ISIN-only Securities link to their issuer
The issuer reading also reads, for a holding with no usable CUSIP, its ISIN
from the pair set and its LEI-shaped issuer LEI; issuer-reduce counts the LEIs
of each ISIN; combine joins the one LEI onto the ISIN Security; the ISIN
Dataset Contract maps ISSUED_BY as the CUSIP one does. Configuration only.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0199JiQoZJ5my5vrS5tW3FQH
</commit_message>
<xml_diff>
--- a/rules/sources/sec.nport.security/MAPPING.xlsx
+++ b/rules/sources/sec.nport.security/MAPPING.xlsx
@@ -638,7 +638,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -910,6 +910,70 @@
       <c r="F9" s="2" t="inlineStr">
         <is>
           <t>mdm.sec.nport.security_isin.v1.contract.adapter.reading.read.tables.mapped.columns.fields.object.fields.issuer_lei</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>sec.nport.security_isin.v1</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>relationship ISSUED_BY</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>to</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>item.issuer_lei</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>Link to gleif.level1.v1</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>mdm.sec.nport.security_isin.v1.contract.adapter.relationships</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>sec.nport.security_isin.v1</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>relationship ISSUED_BY</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>each</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>issuer</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>One link per item (item.)</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>mdm.sec.nport.security_isin.v1.contract.adapter.relationships</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Ticket 102: ISIN-only N-PORT Securities link to their issuer (#1025)
* Ticket 102: ISIN-only Securities link to their issuer

The issuer reading also reads, for a holding with no usable CUSIP, its ISIN
from the pair set and its LEI-shaped issuer LEI; issuer-reduce counts the LEIs
of each ISIN; combine joins the one LEI onto the ISIN Security; the ISIN
Dataset Contract maps ISSUED_BY as the CUSIP one does. Configuration only.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0199JiQoZJ5my5vrS5tW3FQH

* Ticket 102: the real quarter agrees with the direct count

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0199JiQoZJ5my5vrS5tW3FQH

---------

Co-authored-by: Aneena Ananth <aneenaananth@MacBook-Pro.local>
Co-authored-by: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/rules/sources/sec.nport.security/MAPPING.xlsx
+++ b/rules/sources/sec.nport.security/MAPPING.xlsx
@@ -638,7 +638,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -910,6 +910,70 @@
       <c r="F9" s="2" t="inlineStr">
         <is>
           <t>mdm.sec.nport.security_isin.v1.contract.adapter.reading.read.tables.mapped.columns.fields.object.fields.issuer_lei</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>sec.nport.security_isin.v1</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>relationship ISSUED_BY</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>to</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>item.issuer_lei</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>Link to gleif.level1.v1</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>mdm.sec.nport.security_isin.v1.contract.adapter.relationships</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>sec.nport.security_isin.v1</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>relationship ISSUED_BY</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>each</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>issuer</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>One link per item (item.)</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>mdm.sec.nport.security_isin.v1.contract.adapter.relationships</t>
         </is>
       </c>
     </row>

</xml_diff>